<commit_message>
A page for critical gas flow calculations has been added.
</commit_message>
<xml_diff>
--- a/assets/gas_parameters.xlsx
+++ b/assets/gas_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\my-programming\gas-math\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DD78FD-F73A-42F7-8BA0-1F89C98AFA09}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65805B19-D199-42A1-BBD5-C8F904329D0F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="8420" xr2:uid="{E8D457D0-421B-47DB-A602-9D459776E7FE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="184">
   <si>
     <t>Тип</t>
   </si>
@@ -498,30 +498,102 @@
     <t>Температура кипения</t>
   </si>
   <si>
-    <t>Мольная Доля</t>
+    <t>Мольная Доля, %</t>
+  </si>
+  <si>
+    <t>0,02897</t>
+  </si>
+  <si>
+    <t>0,01604</t>
+  </si>
+  <si>
+    <t>0,02604</t>
+  </si>
+  <si>
+    <t>0,02805</t>
+  </si>
+  <si>
+    <t>0,03007</t>
+  </si>
+  <si>
+    <t>0,04208</t>
+  </si>
+  <si>
+    <t>0,0441</t>
+  </si>
+  <si>
+    <t>0,05812</t>
+  </si>
+  <si>
+    <t>0,07215</t>
+  </si>
+  <si>
+    <t>0,08618</t>
+  </si>
+  <si>
+    <t>0,11423</t>
+  </si>
+  <si>
+    <t>0,004</t>
+  </si>
+  <si>
+    <t>0,03995</t>
+  </si>
+  <si>
+    <t>0,02801</t>
+  </si>
+  <si>
+    <t>0,04401</t>
+  </si>
+  <si>
+    <t>0,06406</t>
+  </si>
+  <si>
+    <t>0,04601</t>
+  </si>
+  <si>
+    <t>0,00202</t>
+  </si>
+  <si>
+    <t>0,01801</t>
+  </si>
+  <si>
+    <t>0,01703</t>
+  </si>
+  <si>
+    <t>0,03646</t>
+  </si>
+  <si>
+    <t>0,032</t>
+  </si>
+  <si>
+    <t>0,048</t>
+  </si>
+  <si>
+    <t>0,038</t>
+  </si>
+  <si>
+    <t>0,0709</t>
+  </si>
+  <si>
+    <t>Молярная масса, кг/моль</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="2">
@@ -546,11 +618,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -865,20 +935,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E7EF43C-B293-4564-8C98-2BF91DB98743}">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.90625" customWidth="1"/>
     <col min="2" max="2" width="8.26953125" customWidth="1"/>
     <col min="3" max="3" width="23.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.26953125" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="20.08984375" customWidth="1"/>
     <col min="6" max="6" width="27.36328125" customWidth="1"/>
-    <col min="7" max="7" width="20.6328125" customWidth="1"/>
-    <col min="8" max="8" width="20.08984375" customWidth="1"/>
+    <col min="7" max="7" width="21.1796875" customWidth="1"/>
+    <col min="8" max="8" width="25.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -901,10 +971,13 @@
         <v>155</v>
       </c>
       <c r="H1" t="s">
+        <v>183</v>
+      </c>
+      <c r="O1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -914,23 +987,26 @@
       <c r="C2" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="O2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -940,23 +1016,26 @@
       <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="O3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -966,23 +1045,26 @@
       <c r="C4" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H4" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="O4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -992,23 +1074,26 @@
       <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="H5" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="O5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1018,23 +1103,26 @@
       <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H6" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="O6" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1044,23 +1132,26 @@
       <c r="C7" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>77</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="O7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1070,23 +1161,26 @@
       <c r="C8" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>81</v>
       </c>
       <c r="H8" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="O8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1096,23 +1190,26 @@
       <c r="C9" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="2">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="D9" s="1">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>85</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="O9" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1122,23 +1219,26 @@
       <c r="C10" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>89</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="O10" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1148,23 +1248,26 @@
       <c r="C11" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="2">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="D11" s="1">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>93</v>
       </c>
       <c r="H11" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="O11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1174,23 +1277,26 @@
       <c r="C12" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="s">
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>96</v>
       </c>
       <c r="H12" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="O12" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1200,23 +1306,26 @@
       <c r="C13" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="E13" s="3" t="s">
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>101</v>
       </c>
       <c r="H13" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="O13" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1226,23 +1335,26 @@
       <c r="C14" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>101</v>
       </c>
       <c r="H14" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="O14" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -1252,23 +1364,26 @@
       <c r="C15" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="2">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3" t="s">
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H15" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="O15" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1278,23 +1393,26 @@
       <c r="C16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="2">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="2" t="s">
         <v>112</v>
       </c>
       <c r="H16" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="O16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -1304,23 +1422,26 @@
       <c r="C17" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="2">
-        <v>0</v>
-      </c>
-      <c r="E17" s="3" t="s">
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="2" t="s">
         <v>116</v>
       </c>
       <c r="H17" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="O17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -1330,23 +1451,26 @@
       <c r="C18" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3" t="s">
+      <c r="D18" s="1">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="2" t="s">
         <v>120</v>
       </c>
       <c r="H18" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="O18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -1356,23 +1480,26 @@
       <c r="C19" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="2">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="s">
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="2" t="s">
         <v>124</v>
       </c>
       <c r="H19" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="O19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -1382,23 +1509,26 @@
       <c r="C20" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3" t="s">
+      <c r="D20" s="1">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="2" t="s">
         <v>128</v>
       </c>
       <c r="H20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="O20" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1408,23 +1538,26 @@
       <c r="C21" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="2">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3" t="s">
+      <c r="D21" s="1">
+        <v>0</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="2" t="s">
         <v>61</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="O21" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1434,23 +1567,26 @@
       <c r="C22" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="2">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="D22" s="1">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H22" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="O22" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1460,24 +1596,26 @@
       <c r="C23" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="2">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3" t="s">
+      <c r="D23" s="1">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H23" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="O23" t="s">
         <v>136</v>
       </c>
-      <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -1487,23 +1625,26 @@
       <c r="C24" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3" t="s">
+      <c r="D24" s="1">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H24" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="O24" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -1513,23 +1654,26 @@
       <c r="C25" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="2">
-        <v>0</v>
-      </c>
-      <c r="E25" s="3" t="s">
+      <c r="D25" s="1">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" s="2" t="s">
         <v>116</v>
       </c>
       <c r="H25" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="O25" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -1539,23 +1683,26 @@
       <c r="C26" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="2">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="s">
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="2" t="s">
         <v>108</v>
       </c>
       <c r="H26" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="O26" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -1565,19 +1712,22 @@
       <c r="C27" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="2">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3" t="s">
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="2" t="s">
         <v>148</v>
       </c>
       <c r="H27" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="O27" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
The third list of calculations (flow measuring by a throttle) was added
</commit_message>
<xml_diff>
--- a/assets/gas_parameters.xlsx
+++ b/assets/gas_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\my-programming\gas-math\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65805B19-D199-42A1-BBD5-C8F904329D0F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4BB3AD-FC19-4AD9-A9BD-C1EB5772B0CD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="8420" xr2:uid="{E8D457D0-421B-47DB-A602-9D459776E7FE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="211">
   <si>
     <t>Тип</t>
   </si>
@@ -577,6 +577,87 @@
   </si>
   <si>
     <t>Молярная масса, кг/моль</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>1,10</t>
+  </si>
+  <si>
+    <t>1,02</t>
+  </si>
+  <si>
+    <t>2,04</t>
+  </si>
+  <si>
+    <t>1,01</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>0,80</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>1,96</t>
+  </si>
+  <si>
+    <t>2,24</t>
+  </si>
+  <si>
+    <t>1,75</t>
+  </si>
+  <si>
+    <t>1,47</t>
+  </si>
+  <si>
+    <t>1,26</t>
+  </si>
+  <si>
+    <t>1,32</t>
+  </si>
+  <si>
+    <t>0,88</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>1,44</t>
+  </si>
+  <si>
+    <t>1,76</t>
+  </si>
+  <si>
+    <t>1,34</t>
+  </si>
+  <si>
+    <t>2,28</t>
+  </si>
+  <si>
+    <t>1,33</t>
+  </si>
+  <si>
+    <t>Динамическая вязкость,·10⁻⁵ Па·с</t>
   </si>
 </sst>
 </file>
@@ -616,11 +697,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -946,6 +1028,7 @@
     <col min="6" max="6" width="27.36328125" customWidth="1"/>
     <col min="7" max="7" width="21.1796875" customWidth="1"/>
     <col min="8" max="8" width="25.453125" customWidth="1"/>
+    <col min="9" max="9" width="30.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
@@ -973,6 +1056,9 @@
       <c r="H1" t="s">
         <v>183</v>
       </c>
+      <c r="I1" t="s">
+        <v>210</v>
+      </c>
       <c r="O1" t="s">
         <v>156</v>
       </c>
@@ -1002,6 +1088,9 @@
       <c r="H2" s="3" t="s">
         <v>158</v>
       </c>
+      <c r="I2" s="4" t="s">
+        <v>184</v>
+      </c>
       <c r="O2" t="s">
         <v>152</v>
       </c>
@@ -1031,6 +1120,9 @@
       <c r="H3" s="3" t="s">
         <v>159</v>
       </c>
+      <c r="I3" s="4" t="s">
+        <v>185</v>
+      </c>
       <c r="O3" t="s">
         <v>62</v>
       </c>
@@ -1060,6 +1152,9 @@
       <c r="H4" s="3" t="s">
         <v>160</v>
       </c>
+      <c r="I4" s="4" t="s">
+        <v>186</v>
+      </c>
       <c r="O4" t="s">
         <v>66</v>
       </c>
@@ -1089,6 +1184,9 @@
       <c r="H5" s="3" t="s">
         <v>161</v>
       </c>
+      <c r="I5" s="4" t="s">
+        <v>188</v>
+      </c>
       <c r="O5" t="s">
         <v>70</v>
       </c>
@@ -1118,6 +1216,9 @@
       <c r="H6" s="3" t="s">
         <v>162</v>
       </c>
+      <c r="I6" s="4" t="s">
+        <v>189</v>
+      </c>
       <c r="O6" t="s">
         <v>74</v>
       </c>
@@ -1147,6 +1248,9 @@
       <c r="H7" s="3" t="s">
         <v>163</v>
       </c>
+      <c r="I7" s="4" t="s">
+        <v>190</v>
+      </c>
       <c r="O7" t="s">
         <v>78</v>
       </c>
@@ -1176,6 +1280,9 @@
       <c r="H8" s="3" t="s">
         <v>164</v>
       </c>
+      <c r="I8" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="O8" t="s">
         <v>82</v>
       </c>
@@ -1205,6 +1312,9 @@
       <c r="H9" s="3" t="s">
         <v>165</v>
       </c>
+      <c r="I9" s="4" t="s">
+        <v>192</v>
+      </c>
       <c r="O9" t="s">
         <v>86</v>
       </c>
@@ -1234,6 +1344,9 @@
       <c r="H10" s="3" t="s">
         <v>166</v>
       </c>
+      <c r="I10" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="O10" t="s">
         <v>90</v>
       </c>
@@ -1263,6 +1376,9 @@
       <c r="H11" s="3" t="s">
         <v>167</v>
       </c>
+      <c r="I11" s="4" t="s">
+        <v>194</v>
+      </c>
       <c r="O11" t="s">
         <v>97</v>
       </c>
@@ -1292,6 +1408,9 @@
       <c r="H12" s="3" t="s">
         <v>168</v>
       </c>
+      <c r="I12" s="4" t="s">
+        <v>195</v>
+      </c>
       <c r="O12" t="s">
         <v>98</v>
       </c>
@@ -1321,6 +1440,9 @@
       <c r="H13" s="3" t="s">
         <v>169</v>
       </c>
+      <c r="I13" s="4" t="s">
+        <v>196</v>
+      </c>
       <c r="O13" t="s">
         <v>102</v>
       </c>
@@ -1350,6 +1472,9 @@
       <c r="H14" s="3" t="s">
         <v>170</v>
       </c>
+      <c r="I14" s="4" t="s">
+        <v>197</v>
+      </c>
       <c r="O14" t="s">
         <v>105</v>
       </c>
@@ -1379,6 +1504,9 @@
       <c r="H15" s="3" t="s">
         <v>171</v>
       </c>
+      <c r="I15" s="4" t="s">
+        <v>198</v>
+      </c>
       <c r="O15" t="s">
         <v>109</v>
       </c>
@@ -1408,6 +1536,9 @@
       <c r="H16" s="3" t="s">
         <v>172</v>
       </c>
+      <c r="I16" s="4" t="s">
+        <v>199</v>
+      </c>
       <c r="O16" t="s">
         <v>113</v>
       </c>
@@ -1437,6 +1568,9 @@
       <c r="H17" s="3" t="s">
         <v>173</v>
       </c>
+      <c r="I17" s="4" t="s">
+        <v>200</v>
+      </c>
       <c r="O17" t="s">
         <v>117</v>
       </c>
@@ -1466,6 +1600,9 @@
       <c r="H18" s="3" t="s">
         <v>174</v>
       </c>
+      <c r="I18" s="4" t="s">
+        <v>201</v>
+      </c>
       <c r="O18" t="s">
         <v>121</v>
       </c>
@@ -1495,6 +1632,9 @@
       <c r="H19" s="3" t="s">
         <v>175</v>
       </c>
+      <c r="I19" s="4" t="s">
+        <v>202</v>
+      </c>
       <c r="O19" t="s">
         <v>125</v>
       </c>
@@ -1524,6 +1664,9 @@
       <c r="H20" s="3" t="s">
         <v>176</v>
       </c>
+      <c r="I20" s="4" t="s">
+        <v>203</v>
+      </c>
       <c r="O20" t="s">
         <v>129</v>
       </c>
@@ -1553,6 +1696,9 @@
       <c r="H21" s="3" t="s">
         <v>177</v>
       </c>
+      <c r="I21" s="4" t="s">
+        <v>204</v>
+      </c>
       <c r="O21" t="s">
         <v>132</v>
       </c>
@@ -1582,6 +1728,9 @@
       <c r="H22" s="3" t="s">
         <v>178</v>
       </c>
+      <c r="I22" s="4" t="s">
+        <v>205</v>
+      </c>
       <c r="O22" t="s">
         <v>135</v>
       </c>
@@ -1611,6 +1760,9 @@
       <c r="H23" s="3" t="s">
         <v>171</v>
       </c>
+      <c r="I23" t="s">
+        <v>206</v>
+      </c>
       <c r="O23" t="s">
         <v>136</v>
       </c>
@@ -1640,6 +1792,9 @@
       <c r="H24" s="3" t="s">
         <v>179</v>
       </c>
+      <c r="I24" s="4" t="s">
+        <v>187</v>
+      </c>
       <c r="O24" t="s">
         <v>139</v>
       </c>
@@ -1669,6 +1824,9 @@
       <c r="H25" s="3" t="s">
         <v>180</v>
       </c>
+      <c r="I25" s="4" t="s">
+        <v>207</v>
+      </c>
       <c r="O25" t="s">
         <v>142</v>
       </c>
@@ -1698,6 +1856,9 @@
       <c r="H26" s="3" t="s">
         <v>181</v>
       </c>
+      <c r="I26" s="4" t="s">
+        <v>208</v>
+      </c>
       <c r="O26" t="s">
         <v>145</v>
       </c>
@@ -1726,6 +1887,9 @@
       </c>
       <c r="H27" s="3" t="s">
         <v>182</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>209</v>
       </c>
       <c r="O27" t="s">
         <v>149</v>

</xml_diff>